<commit_message>
Update full complete flowchart
</commit_message>
<xml_diff>
--- a/1.training_model/supplementary/SECTION3.xlsx
+++ b/1.training_model/supplementary/SECTION3.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sitisyaziyah\source\repos\DeviceCluster\1.training_model\supplementary\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD251E22-543A-4194-B8C3-4CCADD661D9C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96B1479B-CA7F-452D-BE6E-DAA19A66784C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="886" xr2:uid="{952F4053-5415-4FB8-A862-7305B9C19CA7}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="886" xr2:uid="{952F4053-5415-4FB8-A862-7305B9C19CA7}"/>
   </bookViews>
   <sheets>
     <sheet name="EXAMPLE" sheetId="13" r:id="rId1"/>
@@ -28,10 +28,10 @@
     <sheet name="section6 - Oiltek " sheetId="8" r:id="rId13"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">EXAMPLE!$D$2:$L$158</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">EXAMPLE!$F$1:$N$157</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'SECTION 5'!$G$2:$H$197</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">SECTION1!$F$2:$N$158</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'section1 - Oiltek'!$B$3:$J$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">SECTION1!$F$1:$N$157</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'section1 - Oiltek'!$A$1:$I$12</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">SECTION2!$G$1:$N$168</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">SECTION3!$E$2:$M$79</definedName>
   </definedNames>
@@ -5319,828 +5319,834 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0E3EE9F4-F0C0-472B-8468-C7661B965326}">
-  <dimension ref="B2:L158"/>
+  <dimension ref="D1:N157"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="12.36328125" customWidth="1"/>
-    <col min="3" max="3" width="8.1796875" customWidth="1"/>
-    <col min="4" max="8" width="10.08984375" bestFit="1" customWidth="1"/>
-    <col min="9" max="11" width="10.36328125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="10.08984375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.36328125" customWidth="1"/>
+    <col min="5" max="5" width="8.1796875" customWidth="1"/>
+    <col min="6" max="6" width="17.1796875" customWidth="1"/>
+    <col min="7" max="7" width="14.1796875" customWidth="1"/>
+    <col min="8" max="8" width="13.54296875" customWidth="1"/>
+    <col min="9" max="9" width="14.1796875" customWidth="1"/>
+    <col min="10" max="10" width="12.453125" customWidth="1"/>
+    <col min="11" max="11" width="12.81640625" customWidth="1"/>
+    <col min="12" max="12" width="12.26953125" customWidth="1"/>
+    <col min="13" max="13" width="11.90625" customWidth="1"/>
+    <col min="14" max="14" width="13.36328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:12" x14ac:dyDescent="0.35">
-      <c r="B2" s="5" t="s">
+    <row r="1" spans="4:14" x14ac:dyDescent="0.35">
+      <c r="D1" s="5" t="s">
         <v>1606</v>
       </c>
-      <c r="C2" s="5" t="s">
+      <c r="E1" s="5" t="s">
         <v>1605</v>
       </c>
-      <c r="D2" s="5" t="s">
+      <c r="F1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="E2" s="5" t="s">
+      <c r="G1" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="F2" s="5" t="s">
+      <c r="H1" s="5" t="s">
         <v>129</v>
       </c>
-      <c r="G2" s="5" t="s">
+      <c r="I1" s="5" t="s">
         <v>185</v>
       </c>
-      <c r="H2" s="5" t="s">
+      <c r="J1" s="5" t="s">
         <v>249</v>
       </c>
-      <c r="I2" s="5" t="s">
+      <c r="K1" s="5" t="s">
         <v>262</v>
       </c>
-      <c r="J2" s="5" t="s">
+      <c r="L1" s="5" t="s">
         <v>265</v>
       </c>
-      <c r="K2" s="5" t="s">
+      <c r="M1" s="5" t="s">
         <v>307</v>
       </c>
-      <c r="L2" s="5" t="s">
+      <c r="N1" s="5" t="s">
         <v>310</v>
       </c>
     </row>
-    <row r="3" spans="2:12" x14ac:dyDescent="0.35">
-      <c r="B3" t="s">
+    <row r="2" spans="4:14" x14ac:dyDescent="0.35">
+      <c r="D2" t="s">
         <v>1152</v>
       </c>
     </row>
-    <row r="4" spans="2:12" x14ac:dyDescent="0.35">
-      <c r="B4" t="s">
+    <row r="3" spans="4:14" x14ac:dyDescent="0.35">
+      <c r="D3" t="s">
         <v>1157</v>
       </c>
     </row>
-    <row r="5" spans="2:12" x14ac:dyDescent="0.35">
-      <c r="B5" t="s">
+    <row r="4" spans="4:14" x14ac:dyDescent="0.35">
+      <c r="D4" t="s">
         <v>1147</v>
       </c>
     </row>
-    <row r="6" spans="2:12" x14ac:dyDescent="0.35">
-      <c r="B6" t="s">
+    <row r="5" spans="4:14" x14ac:dyDescent="0.35">
+      <c r="D5" t="s">
         <v>1142</v>
       </c>
     </row>
-    <row r="7" spans="2:12" x14ac:dyDescent="0.35">
-      <c r="B7" t="s">
+    <row r="6" spans="4:14" x14ac:dyDescent="0.35">
+      <c r="D6" t="s">
         <v>1132</v>
       </c>
     </row>
-    <row r="8" spans="2:12" x14ac:dyDescent="0.35">
-      <c r="B8" t="s">
+    <row r="7" spans="4:14" x14ac:dyDescent="0.35">
+      <c r="D7" t="s">
         <v>1137</v>
       </c>
     </row>
-    <row r="9" spans="2:12" x14ac:dyDescent="0.35">
-      <c r="B9" t="s">
+    <row r="8" spans="4:14" x14ac:dyDescent="0.35">
+      <c r="D8" t="s">
         <v>1162</v>
       </c>
     </row>
-    <row r="10" spans="2:12" x14ac:dyDescent="0.35">
-      <c r="B10" t="s">
+    <row r="9" spans="4:14" x14ac:dyDescent="0.35">
+      <c r="D9" t="s">
         <v>1170</v>
       </c>
     </row>
-    <row r="11" spans="2:12" x14ac:dyDescent="0.35">
-      <c r="B11" t="s">
+    <row r="10" spans="4:14" x14ac:dyDescent="0.35">
+      <c r="D10" t="s">
         <v>1177</v>
       </c>
     </row>
-    <row r="12" spans="2:12" x14ac:dyDescent="0.35">
-      <c r="B12" t="s">
+    <row r="11" spans="4:14" x14ac:dyDescent="0.35">
+      <c r="D11" t="s">
         <v>1183</v>
       </c>
     </row>
-    <row r="13" spans="2:12" x14ac:dyDescent="0.35">
-      <c r="B13" t="s">
+    <row r="12" spans="4:14" x14ac:dyDescent="0.35">
+      <c r="D12" t="s">
         <v>1189</v>
       </c>
     </row>
-    <row r="14" spans="2:12" x14ac:dyDescent="0.35">
-      <c r="B14" t="s">
+    <row r="13" spans="4:14" x14ac:dyDescent="0.35">
+      <c r="D13" t="s">
         <v>1197</v>
       </c>
     </row>
-    <row r="15" spans="2:12" x14ac:dyDescent="0.35">
-      <c r="B15" t="s">
+    <row r="14" spans="4:14" x14ac:dyDescent="0.35">
+      <c r="D14" t="s">
         <v>1204</v>
       </c>
     </row>
-    <row r="16" spans="2:12" x14ac:dyDescent="0.35">
-      <c r="B16" t="s">
+    <row r="15" spans="4:14" x14ac:dyDescent="0.35">
+      <c r="D15" t="s">
         <v>1212</v>
       </c>
     </row>
-    <row r="17" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B17" t="s">
+    <row r="16" spans="4:14" x14ac:dyDescent="0.35">
+      <c r="D16" t="s">
         <v>1219</v>
       </c>
     </row>
-    <row r="18" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B18" t="s">
+    <row r="17" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D17" t="s">
         <v>1225</v>
       </c>
     </row>
-    <row r="19" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B19" t="s">
+    <row r="18" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D18" t="s">
         <v>1233</v>
       </c>
     </row>
-    <row r="20" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B20" t="s">
+    <row r="19" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D19" t="s">
         <v>1240</v>
       </c>
     </row>
-    <row r="21" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B21" t="s">
+    <row r="20" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D20" t="s">
         <v>1246</v>
       </c>
     </row>
-    <row r="22" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B22" t="s">
+    <row r="21" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D21" t="s">
         <v>1254</v>
       </c>
     </row>
-    <row r="23" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B23" t="s">
+    <row r="22" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D22" t="s">
         <v>1261</v>
       </c>
     </row>
-    <row r="24" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B24" t="s">
+    <row r="23" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D23" t="s">
         <v>1267</v>
       </c>
     </row>
-    <row r="25" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B25" t="s">
+    <row r="24" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D24" t="s">
         <v>1275</v>
       </c>
     </row>
-    <row r="26" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B26" t="s">
+    <row r="25" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D25" t="s">
         <v>1282</v>
       </c>
     </row>
-    <row r="27" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B27" t="s">
+    <row r="26" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D26" t="s">
         <v>1163</v>
       </c>
     </row>
-    <row r="28" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B28" t="s">
+    <row r="27" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D27" t="s">
         <v>1171</v>
       </c>
     </row>
-    <row r="29" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B29" t="s">
+    <row r="28" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D28" t="s">
         <v>1190</v>
       </c>
     </row>
-    <row r="30" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B30" t="s">
+    <row r="29" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D29" t="s">
         <v>1198</v>
       </c>
     </row>
-    <row r="31" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B31" t="s">
+    <row r="30" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D30" t="s">
         <v>1205</v>
       </c>
     </row>
-    <row r="32" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B32" t="s">
+    <row r="31" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D31" t="s">
         <v>1213</v>
       </c>
     </row>
-    <row r="33" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B33" t="s">
+    <row r="32" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D32" t="s">
         <v>1226</v>
       </c>
     </row>
-    <row r="34" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B34" t="s">
+    <row r="33" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D33" t="s">
         <v>1234</v>
       </c>
     </row>
-    <row r="35" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B35" t="s">
+    <row r="34" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D34" t="s">
         <v>1247</v>
       </c>
     </row>
-    <row r="36" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B36" t="s">
+    <row r="35" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D35" t="s">
         <v>1255</v>
       </c>
     </row>
-    <row r="37" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B37" t="s">
+    <row r="36" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D36" t="s">
         <v>1268</v>
       </c>
     </row>
-    <row r="38" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B38" t="s">
+    <row r="37" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D37" t="s">
         <v>1276</v>
       </c>
     </row>
-    <row r="39" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B39" t="s">
+    <row r="38" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D38" t="s">
         <v>1164</v>
       </c>
     </row>
-    <row r="40" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B40" t="s">
+    <row r="39" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D39" t="s">
         <v>1172</v>
       </c>
     </row>
-    <row r="41" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B41" t="s">
+    <row r="40" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D40" t="s">
         <v>1178</v>
       </c>
     </row>
-    <row r="42" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B42" t="s">
+    <row r="41" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D41" t="s">
         <v>1184</v>
       </c>
     </row>
-    <row r="43" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B43" t="s">
+    <row r="42" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D42" t="s">
         <v>1191</v>
       </c>
     </row>
-    <row r="44" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B44" t="s">
+    <row r="43" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D43" t="s">
         <v>1199</v>
       </c>
     </row>
-    <row r="45" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B45" t="s">
+    <row r="44" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D44" t="s">
         <v>1206</v>
       </c>
     </row>
-    <row r="46" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B46" t="s">
+    <row r="45" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D45" t="s">
         <v>1214</v>
       </c>
     </row>
-    <row r="47" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B47" t="s">
+    <row r="46" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D46" t="s">
         <v>1220</v>
       </c>
     </row>
-    <row r="48" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B48" t="s">
+    <row r="47" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D47" t="s">
         <v>1227</v>
       </c>
     </row>
-    <row r="49" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B49" t="s">
+    <row r="48" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D48" t="s">
         <v>1235</v>
       </c>
     </row>
-    <row r="50" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B50" t="s">
+    <row r="49" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D49" t="s">
         <v>1241</v>
       </c>
     </row>
-    <row r="51" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B51" t="s">
+    <row r="50" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D50" t="s">
         <v>1248</v>
       </c>
     </row>
-    <row r="52" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B52" t="s">
+    <row r="51" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D51" t="s">
         <v>1256</v>
       </c>
     </row>
-    <row r="53" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B53" t="s">
+    <row r="52" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D52" t="s">
         <v>1262</v>
       </c>
     </row>
-    <row r="54" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B54" t="s">
+    <row r="53" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D53" t="s">
         <v>1269</v>
       </c>
     </row>
-    <row r="55" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B55" t="s">
+    <row r="54" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D54" t="s">
         <v>1277</v>
       </c>
     </row>
-    <row r="56" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B56" t="s">
+    <row r="55" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D55" t="s">
         <v>1283</v>
       </c>
     </row>
-    <row r="57" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B57" t="s">
+    <row r="56" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D56" t="s">
         <v>1153</v>
       </c>
     </row>
-    <row r="58" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B58" t="s">
+    <row r="57" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D57" t="s">
         <v>1158</v>
       </c>
     </row>
-    <row r="59" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B59" t="s">
+    <row r="58" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D58" t="s">
         <v>1148</v>
       </c>
     </row>
-    <row r="60" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B60" t="s">
+    <row r="59" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D59" t="s">
         <v>1143</v>
       </c>
     </row>
-    <row r="61" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B61" t="s">
+    <row r="60" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D60" t="s">
         <v>1133</v>
       </c>
     </row>
-    <row r="62" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B62" t="s">
+    <row r="61" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D61" t="s">
         <v>1138</v>
       </c>
     </row>
-    <row r="63" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B63" t="s">
+    <row r="62" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D62" t="s">
         <v>1165</v>
       </c>
     </row>
-    <row r="64" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B64" t="s">
+    <row r="63" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D63" t="s">
         <v>1173</v>
       </c>
     </row>
-    <row r="65" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B65" t="s">
+    <row r="64" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D64" t="s">
         <v>1179</v>
       </c>
     </row>
-    <row r="66" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B66" t="s">
+    <row r="65" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D65" t="s">
         <v>1185</v>
       </c>
     </row>
-    <row r="67" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B67" t="s">
+    <row r="66" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D66" t="s">
         <v>1192</v>
       </c>
     </row>
-    <row r="68" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B68" t="s">
+    <row r="67" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D67" t="s">
         <v>1200</v>
       </c>
     </row>
-    <row r="69" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B69" t="s">
+    <row r="68" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D68" t="s">
         <v>1207</v>
       </c>
     </row>
-    <row r="70" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B70" t="s">
+    <row r="69" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D69" t="s">
         <v>1215</v>
       </c>
     </row>
-    <row r="71" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B71" t="s">
+    <row r="70" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D70" t="s">
         <v>1221</v>
       </c>
     </row>
-    <row r="72" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B72" t="s">
+    <row r="71" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D71" t="s">
         <v>1228</v>
       </c>
     </row>
-    <row r="73" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B73" t="s">
+    <row r="72" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D72" t="s">
         <v>1236</v>
       </c>
     </row>
-    <row r="74" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B74" t="s">
+    <row r="73" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D73" t="s">
         <v>1242</v>
       </c>
     </row>
-    <row r="75" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B75" t="s">
+    <row r="74" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D74" t="s">
         <v>1249</v>
       </c>
     </row>
-    <row r="76" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B76" t="s">
+    <row r="75" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D75" t="s">
         <v>1257</v>
       </c>
     </row>
-    <row r="77" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B77" t="s">
+    <row r="76" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D76" t="s">
         <v>1263</v>
       </c>
     </row>
-    <row r="78" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B78" t="s">
+    <row r="77" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D77" t="s">
         <v>1270</v>
       </c>
     </row>
-    <row r="79" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B79" t="s">
+    <row r="78" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D78" t="s">
         <v>1278</v>
       </c>
     </row>
-    <row r="80" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B80" t="s">
+    <row r="79" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D79" t="s">
         <v>1284</v>
       </c>
     </row>
-    <row r="81" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B81" t="s">
+    <row r="80" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D80" t="s">
         <v>1166</v>
       </c>
     </row>
-    <row r="82" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B82" t="s">
+    <row r="81" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D81" t="s">
         <v>1193</v>
       </c>
     </row>
-    <row r="83" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B83" t="s">
+    <row r="82" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D82" t="s">
         <v>1208</v>
       </c>
     </row>
-    <row r="84" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B84" t="s">
+    <row r="83" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D83" t="s">
         <v>1229</v>
       </c>
     </row>
-    <row r="85" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B85" t="s">
+    <row r="84" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D84" t="s">
         <v>1250</v>
       </c>
     </row>
-    <row r="86" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B86" t="s">
+    <row r="85" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D85" t="s">
         <v>1271</v>
       </c>
     </row>
-    <row r="87" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B87" t="s">
+    <row r="86" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D86" t="s">
         <v>1167</v>
       </c>
     </row>
-    <row r="88" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B88" t="s">
+    <row r="87" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D87" t="s">
         <v>1174</v>
       </c>
     </row>
-    <row r="89" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B89" t="s">
+    <row r="88" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D88" t="s">
         <v>1180</v>
       </c>
     </row>
-    <row r="90" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B90" t="s">
+    <row r="89" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D89" t="s">
         <v>1186</v>
       </c>
     </row>
-    <row r="91" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B91" t="s">
+    <row r="90" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D90" t="s">
         <v>1194</v>
       </c>
     </row>
-    <row r="92" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B92" t="s">
+    <row r="91" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D91" t="s">
         <v>1201</v>
       </c>
     </row>
-    <row r="93" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B93" t="s">
+    <row r="92" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D92" t="s">
         <v>1209</v>
       </c>
     </row>
-    <row r="94" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B94" t="s">
+    <row r="93" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D93" t="s">
         <v>1216</v>
       </c>
     </row>
-    <row r="95" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B95" t="s">
+    <row r="94" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D94" t="s">
         <v>1222</v>
       </c>
     </row>
-    <row r="96" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B96" t="s">
+    <row r="95" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D95" t="s">
         <v>1230</v>
       </c>
     </row>
-    <row r="97" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B97" t="s">
+    <row r="96" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D96" t="s">
         <v>1237</v>
       </c>
     </row>
-    <row r="98" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B98" t="s">
+    <row r="97" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D97" t="s">
         <v>1243</v>
       </c>
     </row>
-    <row r="99" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B99" t="s">
+    <row r="98" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D98" t="s">
         <v>1251</v>
       </c>
     </row>
-    <row r="100" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B100" t="s">
+    <row r="99" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D99" t="s">
         <v>1258</v>
       </c>
     </row>
-    <row r="101" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B101" t="s">
+    <row r="100" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D100" t="s">
         <v>1264</v>
       </c>
     </row>
-    <row r="102" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B102" t="s">
+    <row r="101" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D101" t="s">
         <v>1272</v>
       </c>
     </row>
-    <row r="103" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B103" t="s">
+    <row r="102" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D102" t="s">
         <v>1279</v>
       </c>
     </row>
-    <row r="104" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B104" t="s">
+    <row r="103" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D103" t="s">
         <v>1285</v>
       </c>
     </row>
-    <row r="105" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B105" t="s">
+    <row r="104" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D104" t="s">
         <v>1168</v>
       </c>
     </row>
-    <row r="106" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B106" t="s">
+    <row r="105" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D105" t="s">
         <v>1175</v>
       </c>
     </row>
-    <row r="107" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B107" t="s">
+    <row r="106" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D106" t="s">
         <v>1181</v>
       </c>
     </row>
-    <row r="108" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B108" t="s">
+    <row r="107" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D107" t="s">
         <v>1187</v>
       </c>
     </row>
-    <row r="109" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B109" t="s">
+    <row r="108" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D108" t="s">
         <v>1195</v>
       </c>
     </row>
-    <row r="110" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B110" t="s">
+    <row r="109" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D109" t="s">
         <v>1202</v>
       </c>
     </row>
-    <row r="111" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B111" t="s">
+    <row r="110" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D110" t="s">
         <v>1210</v>
       </c>
     </row>
-    <row r="112" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B112" t="s">
+    <row r="111" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D111" t="s">
         <v>1217</v>
       </c>
     </row>
-    <row r="113" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B113" t="s">
+    <row r="112" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D112" t="s">
         <v>1223</v>
       </c>
     </row>
-    <row r="114" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B114" t="s">
+    <row r="113" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D113" t="s">
         <v>1231</v>
       </c>
     </row>
-    <row r="115" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B115" t="s">
+    <row r="114" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D114" t="s">
         <v>1238</v>
       </c>
     </row>
-    <row r="116" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B116" t="s">
+    <row r="115" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D115" t="s">
         <v>1244</v>
       </c>
     </row>
-    <row r="117" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B117" t="s">
+    <row r="116" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D116" t="s">
         <v>1252</v>
       </c>
     </row>
-    <row r="118" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B118" t="s">
+    <row r="117" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D117" t="s">
         <v>1259</v>
       </c>
     </row>
-    <row r="119" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B119" t="s">
+    <row r="118" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D118" t="s">
         <v>1265</v>
       </c>
     </row>
-    <row r="120" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B120" t="s">
+    <row r="119" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D119" t="s">
         <v>1273</v>
       </c>
     </row>
-    <row r="121" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B121" t="s">
+    <row r="120" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D120" t="s">
         <v>1280</v>
       </c>
     </row>
-    <row r="122" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B122" t="s">
+    <row r="121" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D121" t="s">
         <v>1286</v>
       </c>
     </row>
-    <row r="123" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B123" t="s">
+    <row r="122" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D122" t="s">
         <v>1154</v>
       </c>
     </row>
-    <row r="124" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B124" t="s">
+    <row r="123" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D123" t="s">
         <v>1159</v>
       </c>
     </row>
-    <row r="125" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B125" t="s">
+    <row r="124" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D124" t="s">
         <v>1149</v>
       </c>
     </row>
-    <row r="126" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B126" t="s">
+    <row r="125" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D125" t="s">
         <v>1144</v>
       </c>
     </row>
-    <row r="127" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B127" t="s">
+    <row r="126" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D126" t="s">
         <v>1134</v>
       </c>
     </row>
-    <row r="128" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B128" t="s">
+    <row r="127" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D127" t="s">
         <v>1139</v>
       </c>
     </row>
-    <row r="129" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B129" t="s">
+    <row r="128" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D128" t="s">
         <v>1155</v>
       </c>
     </row>
-    <row r="130" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B130" t="s">
+    <row r="129" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D129" t="s">
         <v>1160</v>
       </c>
     </row>
-    <row r="131" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B131" t="s">
+    <row r="130" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D130" t="s">
         <v>1150</v>
       </c>
     </row>
-    <row r="132" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B132" t="s">
+    <row r="131" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D131" t="s">
         <v>1145</v>
       </c>
     </row>
-    <row r="133" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B133" t="s">
+    <row r="132" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D132" t="s">
         <v>1135</v>
       </c>
     </row>
-    <row r="134" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B134" t="s">
+    <row r="133" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D133" t="s">
         <v>1140</v>
       </c>
     </row>
-    <row r="135" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B135" t="s">
+    <row r="134" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D134" t="s">
         <v>1169</v>
       </c>
     </row>
-    <row r="136" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B136" t="s">
+    <row r="135" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D135" t="s">
         <v>1176</v>
       </c>
     </row>
-    <row r="137" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B137" t="s">
+    <row r="136" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D136" t="s">
         <v>1182</v>
       </c>
     </row>
-    <row r="138" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B138" t="s">
+    <row r="137" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D137" t="s">
         <v>1188</v>
       </c>
     </row>
-    <row r="139" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B139" t="s">
+    <row r="138" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D138" t="s">
         <v>1196</v>
       </c>
     </row>
-    <row r="140" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B140" t="s">
+    <row r="139" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D139" t="s">
         <v>1203</v>
       </c>
     </row>
-    <row r="141" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B141" t="s">
+    <row r="140" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D140" t="s">
         <v>1211</v>
       </c>
     </row>
-    <row r="142" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B142" t="s">
+    <row r="141" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D141" t="s">
         <v>1218</v>
       </c>
     </row>
-    <row r="143" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B143" t="s">
+    <row r="142" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D142" t="s">
         <v>1224</v>
       </c>
     </row>
-    <row r="144" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B144" t="s">
+    <row r="143" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D143" t="s">
         <v>1232</v>
       </c>
     </row>
-    <row r="145" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B145" t="s">
+    <row r="144" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D144" t="s">
         <v>1239</v>
       </c>
     </row>
-    <row r="146" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B146" t="s">
+    <row r="145" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D145" t="s">
         <v>1245</v>
       </c>
     </row>
-    <row r="147" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B147" t="s">
+    <row r="146" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D146" t="s">
         <v>1253</v>
       </c>
     </row>
-    <row r="148" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B148" t="s">
+    <row r="147" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D147" t="s">
         <v>1260</v>
       </c>
     </row>
-    <row r="149" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B149" t="s">
+    <row r="148" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D148" t="s">
         <v>1266</v>
       </c>
     </row>
-    <row r="150" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B150" t="s">
+    <row r="149" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D149" t="s">
         <v>1274</v>
       </c>
     </row>
-    <row r="151" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B151" t="s">
+    <row r="150" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D150" t="s">
         <v>1281</v>
       </c>
     </row>
-    <row r="152" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B152" t="s">
+    <row r="151" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D151" t="s">
         <v>1287</v>
       </c>
     </row>
-    <row r="153" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B153" t="s">
+    <row r="152" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D152" t="s">
         <v>1156</v>
       </c>
     </row>
-    <row r="154" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B154" t="s">
+    <row r="153" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D153" t="s">
         <v>1161</v>
       </c>
     </row>
-    <row r="155" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B155" t="s">
+    <row r="154" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D154" t="s">
         <v>1151</v>
       </c>
     </row>
-    <row r="156" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B156" t="s">
+    <row r="155" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D155" t="s">
         <v>1146</v>
       </c>
     </row>
-    <row r="157" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B157" t="s">
+    <row r="156" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D156" t="s">
         <v>1136</v>
       </c>
     </row>
-    <row r="158" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B158" t="s">
+    <row r="157" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D157" t="s">
         <v>1141</v>
       </c>
     </row>
@@ -7901,1784 +7907,1790 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{75E7CC39-AA01-4AB9-B162-02F569063FA9}">
-  <dimension ref="F2:N158"/>
+  <dimension ref="F1:N157"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="6" max="10" width="10.08984375" bestFit="1" customWidth="1"/>
-    <col min="11" max="13" width="10.36328125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="10.08984375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.90625" customWidth="1"/>
+    <col min="7" max="7" width="12" customWidth="1"/>
+    <col min="8" max="8" width="12.453125" customWidth="1"/>
+    <col min="9" max="9" width="12" customWidth="1"/>
+    <col min="10" max="10" width="12.54296875" customWidth="1"/>
+    <col min="11" max="11" width="13.81640625" customWidth="1"/>
+    <col min="12" max="12" width="11.7265625" customWidth="1"/>
+    <col min="13" max="13" width="12.7265625" customWidth="1"/>
+    <col min="14" max="14" width="12.81640625" customWidth="1"/>
   </cols>
   <sheetData>
+    <row r="1" spans="6:14" x14ac:dyDescent="0.35">
+      <c r="F1" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="G1" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="H1" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="I1" s="5" t="s">
+        <v>185</v>
+      </c>
+      <c r="J1" s="5" t="s">
+        <v>249</v>
+      </c>
+      <c r="K1" s="5" t="s">
+        <v>262</v>
+      </c>
+      <c r="L1" s="5" t="s">
+        <v>265</v>
+      </c>
+      <c r="M1" s="5" t="s">
+        <v>307</v>
+      </c>
+      <c r="N1" s="5" t="s">
+        <v>310</v>
+      </c>
+    </row>
     <row r="2" spans="6:14" x14ac:dyDescent="0.35">
-      <c r="F2" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="G2" s="5" t="s">
-        <v>78</v>
-      </c>
-      <c r="H2" s="5" t="s">
-        <v>129</v>
-      </c>
-      <c r="I2" s="5" t="s">
-        <v>185</v>
-      </c>
-      <c r="J2" s="5" t="s">
-        <v>249</v>
-      </c>
-      <c r="K2" s="5" t="s">
-        <v>262</v>
-      </c>
-      <c r="L2" s="5" t="s">
-        <v>265</v>
-      </c>
-      <c r="M2" s="5" t="s">
-        <v>307</v>
-      </c>
-      <c r="N2" s="5" t="s">
-        <v>310</v>
+      <c r="F2" t="s">
+        <v>1152</v>
+      </c>
+      <c r="G2" t="s">
+        <v>1308</v>
+      </c>
+      <c r="H2" t="s">
+        <v>1332</v>
+      </c>
+      <c r="I2" t="s">
+        <v>1417</v>
+      </c>
+      <c r="L2" t="s">
+        <v>1492</v>
+      </c>
+      <c r="M2" t="s">
+        <v>1580</v>
+      </c>
+      <c r="N2" t="s">
+        <v>1596</v>
       </c>
     </row>
     <row r="3" spans="6:14" x14ac:dyDescent="0.35">
       <c r="F3" t="s">
-        <v>1152</v>
-      </c>
-      <c r="G3" t="s">
-        <v>1308</v>
+        <v>1157</v>
       </c>
       <c r="H3" t="s">
-        <v>1332</v>
+        <v>1337</v>
       </c>
       <c r="I3" t="s">
-        <v>1417</v>
+        <v>1422</v>
       </c>
       <c r="L3" t="s">
-        <v>1492</v>
-      </c>
-      <c r="M3" t="s">
-        <v>1580</v>
-      </c>
-      <c r="N3" t="s">
-        <v>1596</v>
+        <v>1497</v>
       </c>
     </row>
     <row r="4" spans="6:14" x14ac:dyDescent="0.35">
       <c r="F4" t="s">
-        <v>1157</v>
+        <v>1147</v>
+      </c>
+      <c r="G4" t="s">
+        <v>1303</v>
       </c>
       <c r="H4" t="s">
-        <v>1337</v>
+        <v>1327</v>
       </c>
       <c r="I4" t="s">
-        <v>1422</v>
+        <v>1412</v>
       </c>
       <c r="L4" t="s">
-        <v>1497</v>
+        <v>1487</v>
+      </c>
+      <c r="M4" t="s">
+        <v>1575</v>
+      </c>
+      <c r="N4" t="s">
+        <v>1591</v>
       </c>
     </row>
     <row r="5" spans="6:14" x14ac:dyDescent="0.35">
       <c r="F5" t="s">
-        <v>1147</v>
+        <v>1142</v>
       </c>
       <c r="G5" t="s">
-        <v>1303</v>
+        <v>1298</v>
       </c>
       <c r="H5" t="s">
-        <v>1327</v>
+        <v>1322</v>
       </c>
       <c r="I5" t="s">
-        <v>1412</v>
+        <v>1407</v>
+      </c>
+      <c r="J5" t="s">
+        <v>1460</v>
       </c>
       <c r="L5" t="s">
-        <v>1487</v>
+        <v>1482</v>
       </c>
       <c r="M5" t="s">
-        <v>1575</v>
+        <v>1570</v>
       </c>
       <c r="N5" t="s">
-        <v>1591</v>
+        <v>1201</v>
       </c>
     </row>
     <row r="6" spans="6:14" x14ac:dyDescent="0.35">
       <c r="F6" t="s">
-        <v>1142</v>
+        <v>1132</v>
       </c>
       <c r="G6" t="s">
-        <v>1298</v>
+        <v>1288</v>
       </c>
       <c r="H6" t="s">
-        <v>1322</v>
+        <v>1312</v>
       </c>
       <c r="I6" t="s">
-        <v>1407</v>
+        <v>1397</v>
       </c>
       <c r="J6" t="s">
-        <v>1460</v>
+        <v>1450</v>
+      </c>
+      <c r="K6" t="s">
+        <v>1465</v>
       </c>
       <c r="L6" t="s">
-        <v>1482</v>
+        <v>1472</v>
       </c>
       <c r="M6" t="s">
-        <v>1570</v>
+        <v>1560</v>
       </c>
       <c r="N6" t="s">
-        <v>1201</v>
+        <v>1585</v>
       </c>
     </row>
     <row r="7" spans="6:14" x14ac:dyDescent="0.35">
       <c r="F7" t="s">
-        <v>1132</v>
+        <v>1137</v>
       </c>
       <c r="G7" t="s">
-        <v>1288</v>
+        <v>1293</v>
       </c>
       <c r="H7" t="s">
-        <v>1312</v>
+        <v>1317</v>
       </c>
       <c r="I7" t="s">
-        <v>1397</v>
+        <v>1402</v>
       </c>
       <c r="J7" t="s">
-        <v>1450</v>
+        <v>1455</v>
       </c>
       <c r="K7" t="s">
-        <v>1465</v>
+        <v>1470</v>
       </c>
       <c r="L7" t="s">
-        <v>1472</v>
+        <v>1477</v>
       </c>
       <c r="M7" t="s">
-        <v>1560</v>
+        <v>1565</v>
       </c>
       <c r="N7" t="s">
-        <v>1585</v>
+        <v>1192</v>
       </c>
     </row>
     <row r="8" spans="6:14" x14ac:dyDescent="0.35">
       <c r="F8" t="s">
-        <v>1137</v>
-      </c>
-      <c r="G8" t="s">
-        <v>1293</v>
+        <v>1162</v>
       </c>
       <c r="H8" t="s">
-        <v>1317</v>
+        <v>1342</v>
       </c>
       <c r="I8" t="s">
-        <v>1402</v>
-      </c>
-      <c r="J8" t="s">
-        <v>1455</v>
-      </c>
-      <c r="K8" t="s">
-        <v>1470</v>
+        <v>1427</v>
       </c>
       <c r="L8" t="s">
-        <v>1477</v>
-      </c>
-      <c r="M8" t="s">
-        <v>1565</v>
-      </c>
-      <c r="N8" t="s">
-        <v>1192</v>
+        <v>1502</v>
       </c>
     </row>
     <row r="9" spans="6:14" x14ac:dyDescent="0.35">
       <c r="F9" t="s">
-        <v>1162</v>
+        <v>1170</v>
       </c>
       <c r="H9" t="s">
-        <v>1342</v>
+        <v>1350</v>
       </c>
       <c r="I9" t="s">
-        <v>1427</v>
+        <v>1435</v>
       </c>
       <c r="L9" t="s">
-        <v>1502</v>
+        <v>1510</v>
       </c>
     </row>
     <row r="10" spans="6:14" x14ac:dyDescent="0.35">
       <c r="F10" t="s">
-        <v>1170</v>
+        <v>1177</v>
       </c>
       <c r="H10" t="s">
-        <v>1350</v>
+        <v>1357</v>
       </c>
       <c r="I10" t="s">
-        <v>1435</v>
+        <v>1442</v>
       </c>
       <c r="L10" t="s">
-        <v>1510</v>
+        <v>1517</v>
       </c>
     </row>
     <row r="11" spans="6:14" x14ac:dyDescent="0.35">
       <c r="F11" t="s">
-        <v>1177</v>
+        <v>1183</v>
       </c>
       <c r="H11" t="s">
-        <v>1357</v>
+        <v>1363</v>
       </c>
       <c r="I11" t="s">
-        <v>1442</v>
+        <v>1448</v>
       </c>
       <c r="L11" t="s">
-        <v>1517</v>
+        <v>1523</v>
       </c>
     </row>
     <row r="12" spans="6:14" x14ac:dyDescent="0.35">
       <c r="F12" t="s">
-        <v>1183</v>
+        <v>1189</v>
       </c>
       <c r="H12" t="s">
-        <v>1363</v>
-      </c>
-      <c r="I12" t="s">
-        <v>1448</v>
+        <v>1369</v>
       </c>
       <c r="L12" t="s">
-        <v>1523</v>
+        <v>1529</v>
       </c>
     </row>
     <row r="13" spans="6:14" x14ac:dyDescent="0.35">
       <c r="F13" t="s">
-        <v>1189</v>
+        <v>1197</v>
       </c>
       <c r="H13" t="s">
-        <v>1369</v>
+        <v>1377</v>
       </c>
       <c r="L13" t="s">
-        <v>1529</v>
+        <v>1537</v>
       </c>
     </row>
     <row r="14" spans="6:14" x14ac:dyDescent="0.35">
       <c r="F14" t="s">
-        <v>1197</v>
+        <v>1204</v>
       </c>
       <c r="H14" t="s">
-        <v>1377</v>
+        <v>1384</v>
       </c>
       <c r="L14" t="s">
-        <v>1537</v>
+        <v>1544</v>
       </c>
     </row>
     <row r="15" spans="6:14" x14ac:dyDescent="0.35">
       <c r="F15" t="s">
-        <v>1204</v>
+        <v>1212</v>
       </c>
       <c r="H15" t="s">
-        <v>1384</v>
+        <v>1392</v>
       </c>
       <c r="L15" t="s">
-        <v>1544</v>
+        <v>1552</v>
       </c>
     </row>
     <row r="16" spans="6:14" x14ac:dyDescent="0.35">
       <c r="F16" t="s">
-        <v>1212</v>
-      </c>
-      <c r="H16" t="s">
-        <v>1392</v>
+        <v>1219</v>
       </c>
       <c r="L16" t="s">
-        <v>1552</v>
+        <v>1559</v>
       </c>
     </row>
     <row r="17" spans="6:12" x14ac:dyDescent="0.35">
       <c r="F17" t="s">
-        <v>1219</v>
-      </c>
-      <c r="L17" t="s">
-        <v>1559</v>
+        <v>1225</v>
       </c>
     </row>
     <row r="18" spans="6:12" x14ac:dyDescent="0.35">
       <c r="F18" t="s">
-        <v>1225</v>
+        <v>1233</v>
       </c>
     </row>
     <row r="19" spans="6:12" x14ac:dyDescent="0.35">
       <c r="F19" t="s">
-        <v>1233</v>
+        <v>1240</v>
       </c>
     </row>
     <row r="20" spans="6:12" x14ac:dyDescent="0.35">
       <c r="F20" t="s">
-        <v>1240</v>
+        <v>1246</v>
       </c>
     </row>
     <row r="21" spans="6:12" x14ac:dyDescent="0.35">
       <c r="F21" t="s">
-        <v>1246</v>
+        <v>1254</v>
       </c>
     </row>
     <row r="22" spans="6:12" x14ac:dyDescent="0.35">
       <c r="F22" t="s">
-        <v>1254</v>
+        <v>1261</v>
       </c>
     </row>
     <row r="23" spans="6:12" x14ac:dyDescent="0.35">
       <c r="F23" t="s">
-        <v>1261</v>
+        <v>1267</v>
       </c>
     </row>
     <row r="24" spans="6:12" x14ac:dyDescent="0.35">
       <c r="F24" t="s">
-        <v>1267</v>
+        <v>1275</v>
       </c>
     </row>
     <row r="25" spans="6:12" x14ac:dyDescent="0.35">
       <c r="F25" t="s">
-        <v>1275</v>
+        <v>1282</v>
       </c>
     </row>
     <row r="26" spans="6:12" x14ac:dyDescent="0.35">
       <c r="F26" t="s">
-        <v>1282</v>
+        <v>1163</v>
+      </c>
+      <c r="H26" t="s">
+        <v>1343</v>
+      </c>
+      <c r="I26" t="s">
+        <v>1428</v>
+      </c>
+      <c r="L26" t="s">
+        <v>1503</v>
       </c>
     </row>
     <row r="27" spans="6:12" x14ac:dyDescent="0.35">
       <c r="F27" t="s">
-        <v>1163</v>
+        <v>1171</v>
       </c>
       <c r="H27" t="s">
-        <v>1343</v>
+        <v>1351</v>
       </c>
       <c r="I27" t="s">
-        <v>1428</v>
+        <v>1436</v>
       </c>
       <c r="L27" t="s">
-        <v>1503</v>
+        <v>1511</v>
       </c>
     </row>
     <row r="28" spans="6:12" x14ac:dyDescent="0.35">
       <c r="F28" t="s">
-        <v>1171</v>
+        <v>1190</v>
       </c>
       <c r="H28" t="s">
-        <v>1351</v>
-      </c>
-      <c r="I28" t="s">
-        <v>1436</v>
+        <v>1370</v>
       </c>
       <c r="L28" t="s">
-        <v>1511</v>
+        <v>1530</v>
       </c>
     </row>
     <row r="29" spans="6:12" x14ac:dyDescent="0.35">
       <c r="F29" t="s">
-        <v>1190</v>
+        <v>1198</v>
       </c>
       <c r="H29" t="s">
-        <v>1370</v>
+        <v>1378</v>
       </c>
       <c r="L29" t="s">
-        <v>1530</v>
+        <v>1538</v>
       </c>
     </row>
     <row r="30" spans="6:12" x14ac:dyDescent="0.35">
       <c r="F30" t="s">
-        <v>1198</v>
+        <v>1205</v>
       </c>
       <c r="H30" t="s">
-        <v>1378</v>
+        <v>1385</v>
       </c>
       <c r="L30" t="s">
-        <v>1538</v>
+        <v>1545</v>
       </c>
     </row>
     <row r="31" spans="6:12" x14ac:dyDescent="0.35">
       <c r="F31" t="s">
-        <v>1205</v>
+        <v>1213</v>
       </c>
       <c r="H31" t="s">
-        <v>1385</v>
+        <v>1393</v>
       </c>
       <c r="L31" t="s">
-        <v>1545</v>
+        <v>1553</v>
       </c>
     </row>
     <row r="32" spans="6:12" x14ac:dyDescent="0.35">
       <c r="F32" t="s">
-        <v>1213</v>
-      </c>
-      <c r="H32" t="s">
-        <v>1393</v>
-      </c>
-      <c r="L32" t="s">
-        <v>1553</v>
+        <v>1226</v>
       </c>
     </row>
     <row r="33" spans="6:12" x14ac:dyDescent="0.35">
       <c r="F33" t="s">
-        <v>1226</v>
+        <v>1234</v>
       </c>
     </row>
     <row r="34" spans="6:12" x14ac:dyDescent="0.35">
       <c r="F34" t="s">
-        <v>1234</v>
+        <v>1247</v>
       </c>
     </row>
     <row r="35" spans="6:12" x14ac:dyDescent="0.35">
       <c r="F35" t="s">
-        <v>1247</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="36" spans="6:12" x14ac:dyDescent="0.35">
       <c r="F36" t="s">
-        <v>1255</v>
+        <v>1268</v>
       </c>
     </row>
     <row r="37" spans="6:12" x14ac:dyDescent="0.35">
       <c r="F37" t="s">
-        <v>1268</v>
+        <v>1276</v>
       </c>
     </row>
     <row r="38" spans="6:12" x14ac:dyDescent="0.35">
       <c r="F38" t="s">
-        <v>1276</v>
+        <v>1164</v>
+      </c>
+      <c r="H38" t="s">
+        <v>1344</v>
+      </c>
+      <c r="I38" t="s">
+        <v>1429</v>
+      </c>
+      <c r="L38" t="s">
+        <v>1504</v>
       </c>
     </row>
     <row r="39" spans="6:12" x14ac:dyDescent="0.35">
       <c r="F39" t="s">
-        <v>1164</v>
+        <v>1172</v>
       </c>
       <c r="H39" t="s">
-        <v>1344</v>
+        <v>1352</v>
       </c>
       <c r="I39" t="s">
-        <v>1429</v>
+        <v>1437</v>
       </c>
       <c r="L39" t="s">
-        <v>1504</v>
+        <v>1512</v>
       </c>
     </row>
     <row r="40" spans="6:12" x14ac:dyDescent="0.35">
       <c r="F40" t="s">
-        <v>1172</v>
+        <v>1178</v>
       </c>
       <c r="H40" t="s">
-        <v>1352</v>
+        <v>1358</v>
       </c>
       <c r="I40" t="s">
-        <v>1437</v>
+        <v>1443</v>
       </c>
       <c r="L40" t="s">
-        <v>1512</v>
+        <v>1518</v>
       </c>
     </row>
     <row r="41" spans="6:12" x14ac:dyDescent="0.35">
       <c r="F41" t="s">
-        <v>1178</v>
+        <v>1184</v>
       </c>
       <c r="H41" t="s">
-        <v>1358</v>
+        <v>1364</v>
       </c>
       <c r="I41" t="s">
-        <v>1443</v>
+        <v>1449</v>
       </c>
       <c r="L41" t="s">
-        <v>1518</v>
+        <v>1524</v>
       </c>
     </row>
     <row r="42" spans="6:12" x14ac:dyDescent="0.35">
       <c r="F42" t="s">
-        <v>1184</v>
+        <v>1191</v>
       </c>
       <c r="H42" t="s">
-        <v>1364</v>
-      </c>
-      <c r="I42" t="s">
-        <v>1449</v>
+        <v>1371</v>
       </c>
       <c r="L42" t="s">
-        <v>1524</v>
+        <v>1531</v>
       </c>
     </row>
     <row r="43" spans="6:12" x14ac:dyDescent="0.35">
       <c r="F43" t="s">
-        <v>1191</v>
+        <v>1199</v>
       </c>
       <c r="H43" t="s">
-        <v>1371</v>
+        <v>1379</v>
       </c>
       <c r="L43" t="s">
-        <v>1531</v>
+        <v>1539</v>
       </c>
     </row>
     <row r="44" spans="6:12" x14ac:dyDescent="0.35">
       <c r="F44" t="s">
-        <v>1199</v>
+        <v>1206</v>
       </c>
       <c r="H44" t="s">
-        <v>1379</v>
+        <v>1386</v>
       </c>
       <c r="L44" t="s">
-        <v>1539</v>
+        <v>1546</v>
       </c>
     </row>
     <row r="45" spans="6:12" x14ac:dyDescent="0.35">
       <c r="F45" t="s">
-        <v>1206</v>
+        <v>1214</v>
       </c>
       <c r="H45" t="s">
-        <v>1386</v>
+        <v>1394</v>
       </c>
       <c r="L45" t="s">
-        <v>1546</v>
+        <v>1554</v>
       </c>
     </row>
     <row r="46" spans="6:12" x14ac:dyDescent="0.35">
       <c r="F46" t="s">
-        <v>1214</v>
-      </c>
-      <c r="H46" t="s">
-        <v>1394</v>
-      </c>
-      <c r="L46" t="s">
-        <v>1554</v>
+        <v>1220</v>
       </c>
     </row>
     <row r="47" spans="6:12" x14ac:dyDescent="0.35">
       <c r="F47" t="s">
-        <v>1220</v>
+        <v>1227</v>
       </c>
     </row>
     <row r="48" spans="6:12" x14ac:dyDescent="0.35">
       <c r="F48" t="s">
-        <v>1227</v>
+        <v>1235</v>
       </c>
     </row>
     <row r="49" spans="6:14" x14ac:dyDescent="0.35">
       <c r="F49" t="s">
-        <v>1235</v>
+        <v>1241</v>
       </c>
     </row>
     <row r="50" spans="6:14" x14ac:dyDescent="0.35">
       <c r="F50" t="s">
-        <v>1241</v>
+        <v>1248</v>
       </c>
     </row>
     <row r="51" spans="6:14" x14ac:dyDescent="0.35">
       <c r="F51" t="s">
-        <v>1248</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="52" spans="6:14" x14ac:dyDescent="0.35">
       <c r="F52" t="s">
-        <v>1256</v>
+        <v>1262</v>
       </c>
     </row>
     <row r="53" spans="6:14" x14ac:dyDescent="0.35">
       <c r="F53" t="s">
-        <v>1262</v>
+        <v>1269</v>
       </c>
     </row>
     <row r="54" spans="6:14" x14ac:dyDescent="0.35">
       <c r="F54" t="s">
-        <v>1269</v>
+        <v>1277</v>
       </c>
     </row>
     <row r="55" spans="6:14" x14ac:dyDescent="0.35">
       <c r="F55" t="s">
-        <v>1277</v>
+        <v>1283</v>
       </c>
     </row>
     <row r="56" spans="6:14" x14ac:dyDescent="0.35">
       <c r="F56" t="s">
-        <v>1283</v>
+        <v>1153</v>
+      </c>
+      <c r="G56" t="s">
+        <v>1309</v>
+      </c>
+      <c r="H56" t="s">
+        <v>1333</v>
+      </c>
+      <c r="I56" t="s">
+        <v>1418</v>
+      </c>
+      <c r="L56" t="s">
+        <v>1493</v>
+      </c>
+      <c r="M56" t="s">
+        <v>1581</v>
+      </c>
+      <c r="N56" t="s">
+        <v>1597</v>
       </c>
     </row>
     <row r="57" spans="6:14" x14ac:dyDescent="0.35">
       <c r="F57" t="s">
-        <v>1153</v>
-      </c>
-      <c r="G57" t="s">
-        <v>1309</v>
+        <v>1158</v>
       </c>
       <c r="H57" t="s">
-        <v>1333</v>
+        <v>1338</v>
       </c>
       <c r="I57" t="s">
-        <v>1418</v>
+        <v>1423</v>
       </c>
       <c r="L57" t="s">
-        <v>1493</v>
-      </c>
-      <c r="M57" t="s">
-        <v>1581</v>
-      </c>
-      <c r="N57" t="s">
-        <v>1597</v>
+        <v>1498</v>
       </c>
     </row>
     <row r="58" spans="6:14" x14ac:dyDescent="0.35">
       <c r="F58" t="s">
-        <v>1158</v>
+        <v>1148</v>
+      </c>
+      <c r="G58" t="s">
+        <v>1304</v>
       </c>
       <c r="H58" t="s">
-        <v>1338</v>
+        <v>1328</v>
       </c>
       <c r="I58" t="s">
-        <v>1423</v>
+        <v>1413</v>
       </c>
       <c r="L58" t="s">
-        <v>1498</v>
+        <v>1488</v>
+      </c>
+      <c r="M58" t="s">
+        <v>1576</v>
+      </c>
+      <c r="N58" t="s">
+        <v>1592</v>
       </c>
     </row>
     <row r="59" spans="6:14" x14ac:dyDescent="0.35">
       <c r="F59" t="s">
-        <v>1148</v>
+        <v>1143</v>
       </c>
       <c r="G59" t="s">
-        <v>1304</v>
+        <v>1299</v>
       </c>
       <c r="H59" t="s">
-        <v>1328</v>
+        <v>1323</v>
       </c>
       <c r="I59" t="s">
-        <v>1413</v>
+        <v>1408</v>
+      </c>
+      <c r="J59" t="s">
+        <v>1461</v>
       </c>
       <c r="L59" t="s">
-        <v>1488</v>
+        <v>1483</v>
       </c>
       <c r="M59" t="s">
-        <v>1576</v>
+        <v>1571</v>
       </c>
       <c r="N59" t="s">
-        <v>1592</v>
+        <v>1202</v>
       </c>
     </row>
     <row r="60" spans="6:14" x14ac:dyDescent="0.35">
       <c r="F60" t="s">
-        <v>1143</v>
+        <v>1133</v>
       </c>
       <c r="G60" t="s">
-        <v>1299</v>
+        <v>1289</v>
       </c>
       <c r="H60" t="s">
-        <v>1323</v>
+        <v>1313</v>
       </c>
       <c r="I60" t="s">
-        <v>1408</v>
+        <v>1398</v>
       </c>
       <c r="J60" t="s">
-        <v>1461</v>
+        <v>1451</v>
+      </c>
+      <c r="K60" t="s">
+        <v>1466</v>
       </c>
       <c r="L60" t="s">
-        <v>1483</v>
+        <v>1473</v>
       </c>
       <c r="M60" t="s">
-        <v>1571</v>
+        <v>1561</v>
       </c>
       <c r="N60" t="s">
-        <v>1202</v>
+        <v>1586</v>
       </c>
     </row>
     <row r="61" spans="6:14" x14ac:dyDescent="0.35">
       <c r="F61" t="s">
-        <v>1133</v>
+        <v>1138</v>
       </c>
       <c r="G61" t="s">
-        <v>1289</v>
+        <v>1294</v>
       </c>
       <c r="H61" t="s">
-        <v>1313</v>
+        <v>1318</v>
       </c>
       <c r="I61" t="s">
-        <v>1398</v>
+        <v>1403</v>
       </c>
       <c r="J61" t="s">
-        <v>1451</v>
+        <v>1456</v>
       </c>
       <c r="K61" t="s">
-        <v>1466</v>
+        <v>1471</v>
       </c>
       <c r="L61" t="s">
-        <v>1473</v>
+        <v>1478</v>
       </c>
       <c r="M61" t="s">
-        <v>1561</v>
+        <v>1566</v>
       </c>
       <c r="N61" t="s">
-        <v>1586</v>
+        <v>1587</v>
       </c>
     </row>
     <row r="62" spans="6:14" x14ac:dyDescent="0.35">
       <c r="F62" t="s">
-        <v>1138</v>
-      </c>
-      <c r="G62" t="s">
-        <v>1294</v>
+        <v>1165</v>
       </c>
       <c r="H62" t="s">
-        <v>1318</v>
+        <v>1345</v>
       </c>
       <c r="I62" t="s">
-        <v>1403</v>
-      </c>
-      <c r="J62" t="s">
-        <v>1456</v>
-      </c>
-      <c r="K62" t="s">
-        <v>1471</v>
+        <v>1430</v>
       </c>
       <c r="L62" t="s">
-        <v>1478</v>
-      </c>
-      <c r="M62" t="s">
-        <v>1566</v>
-      </c>
-      <c r="N62" t="s">
-        <v>1587</v>
+        <v>1505</v>
       </c>
     </row>
     <row r="63" spans="6:14" x14ac:dyDescent="0.35">
       <c r="F63" t="s">
-        <v>1165</v>
+        <v>1173</v>
       </c>
       <c r="H63" t="s">
-        <v>1345</v>
+        <v>1353</v>
       </c>
       <c r="I63" t="s">
-        <v>1430</v>
+        <v>1438</v>
       </c>
       <c r="L63" t="s">
-        <v>1505</v>
+        <v>1513</v>
       </c>
     </row>
     <row r="64" spans="6:14" x14ac:dyDescent="0.35">
       <c r="F64" t="s">
-        <v>1173</v>
+        <v>1179</v>
       </c>
       <c r="H64" t="s">
-        <v>1353</v>
+        <v>1359</v>
       </c>
       <c r="I64" t="s">
-        <v>1438</v>
+        <v>1444</v>
       </c>
       <c r="L64" t="s">
-        <v>1513</v>
+        <v>1519</v>
       </c>
     </row>
     <row r="65" spans="6:12" x14ac:dyDescent="0.35">
       <c r="F65" t="s">
-        <v>1179</v>
+        <v>1185</v>
       </c>
       <c r="H65" t="s">
-        <v>1359</v>
-      </c>
-      <c r="I65" t="s">
-        <v>1444</v>
+        <v>1365</v>
       </c>
       <c r="L65" t="s">
-        <v>1519</v>
+        <v>1525</v>
       </c>
     </row>
     <row r="66" spans="6:12" x14ac:dyDescent="0.35">
       <c r="F66" t="s">
-        <v>1185</v>
+        <v>1192</v>
       </c>
       <c r="H66" t="s">
-        <v>1365</v>
+        <v>1372</v>
       </c>
       <c r="L66" t="s">
-        <v>1525</v>
+        <v>1532</v>
       </c>
     </row>
     <row r="67" spans="6:12" x14ac:dyDescent="0.35">
       <c r="F67" t="s">
-        <v>1192</v>
+        <v>1200</v>
       </c>
       <c r="H67" t="s">
-        <v>1372</v>
+        <v>1380</v>
       </c>
       <c r="L67" t="s">
-        <v>1532</v>
+        <v>1540</v>
       </c>
     </row>
     <row r="68" spans="6:12" x14ac:dyDescent="0.35">
       <c r="F68" t="s">
-        <v>1200</v>
+        <v>1207</v>
       </c>
       <c r="H68" t="s">
-        <v>1380</v>
+        <v>1387</v>
       </c>
       <c r="L68" t="s">
-        <v>1540</v>
+        <v>1547</v>
       </c>
     </row>
     <row r="69" spans="6:12" x14ac:dyDescent="0.35">
       <c r="F69" t="s">
-        <v>1207</v>
+        <v>1215</v>
       </c>
       <c r="H69" t="s">
-        <v>1387</v>
+        <v>1395</v>
       </c>
       <c r="L69" t="s">
-        <v>1547</v>
+        <v>1555</v>
       </c>
     </row>
     <row r="70" spans="6:12" x14ac:dyDescent="0.35">
       <c r="F70" t="s">
-        <v>1215</v>
-      </c>
-      <c r="H70" t="s">
-        <v>1395</v>
-      </c>
-      <c r="L70" t="s">
-        <v>1555</v>
+        <v>1221</v>
       </c>
     </row>
     <row r="71" spans="6:12" x14ac:dyDescent="0.35">
       <c r="F71" t="s">
-        <v>1221</v>
+        <v>1228</v>
       </c>
     </row>
     <row r="72" spans="6:12" x14ac:dyDescent="0.35">
       <c r="F72" t="s">
-        <v>1228</v>
+        <v>1236</v>
       </c>
     </row>
     <row r="73" spans="6:12" x14ac:dyDescent="0.35">
       <c r="F73" t="s">
-        <v>1236</v>
+        <v>1242</v>
       </c>
     </row>
     <row r="74" spans="6:12" x14ac:dyDescent="0.35">
       <c r="F74" t="s">
-        <v>1242</v>
+        <v>1249</v>
       </c>
     </row>
     <row r="75" spans="6:12" x14ac:dyDescent="0.35">
       <c r="F75" t="s">
-        <v>1249</v>
+        <v>1257</v>
       </c>
     </row>
     <row r="76" spans="6:12" x14ac:dyDescent="0.35">
       <c r="F76" t="s">
-        <v>1257</v>
+        <v>1263</v>
       </c>
     </row>
     <row r="77" spans="6:12" x14ac:dyDescent="0.35">
       <c r="F77" t="s">
-        <v>1263</v>
+        <v>1270</v>
       </c>
     </row>
     <row r="78" spans="6:12" x14ac:dyDescent="0.35">
       <c r="F78" t="s">
-        <v>1270</v>
+        <v>1278</v>
       </c>
     </row>
     <row r="79" spans="6:12" x14ac:dyDescent="0.35">
       <c r="F79" t="s">
-        <v>1278</v>
+        <v>1284</v>
       </c>
     </row>
     <row r="80" spans="6:12" x14ac:dyDescent="0.35">
       <c r="F80" t="s">
-        <v>1284</v>
+        <v>1166</v>
+      </c>
+      <c r="H80" t="s">
+        <v>1346</v>
+      </c>
+      <c r="I80" t="s">
+        <v>1431</v>
+      </c>
+      <c r="L80" t="s">
+        <v>1506</v>
       </c>
     </row>
     <row r="81" spans="6:12" x14ac:dyDescent="0.35">
       <c r="F81" t="s">
-        <v>1166</v>
+        <v>1193</v>
       </c>
       <c r="H81" t="s">
-        <v>1346</v>
-      </c>
-      <c r="I81" t="s">
-        <v>1431</v>
+        <v>1373</v>
       </c>
       <c r="L81" t="s">
-        <v>1506</v>
+        <v>1533</v>
       </c>
     </row>
     <row r="82" spans="6:12" x14ac:dyDescent="0.35">
       <c r="F82" t="s">
-        <v>1193</v>
+        <v>1208</v>
       </c>
       <c r="H82" t="s">
-        <v>1373</v>
+        <v>1388</v>
       </c>
       <c r="L82" t="s">
-        <v>1533</v>
+        <v>1548</v>
       </c>
     </row>
     <row r="83" spans="6:12" x14ac:dyDescent="0.35">
       <c r="F83" t="s">
-        <v>1208</v>
-      </c>
-      <c r="H83" t="s">
-        <v>1388</v>
-      </c>
-      <c r="L83" t="s">
-        <v>1548</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="84" spans="6:12" x14ac:dyDescent="0.35">
       <c r="F84" t="s">
-        <v>1229</v>
+        <v>1250</v>
       </c>
     </row>
     <row r="85" spans="6:12" x14ac:dyDescent="0.35">
       <c r="F85" t="s">
-        <v>1250</v>
+        <v>1271</v>
       </c>
     </row>
     <row r="86" spans="6:12" x14ac:dyDescent="0.35">
       <c r="F86" t="s">
-        <v>1271</v>
+        <v>1167</v>
+      </c>
+      <c r="H86" t="s">
+        <v>1347</v>
+      </c>
+      <c r="I86" t="s">
+        <v>1432</v>
+      </c>
+      <c r="L86" t="s">
+        <v>1507</v>
       </c>
     </row>
     <row r="87" spans="6:12" x14ac:dyDescent="0.35">
       <c r="F87" t="s">
-        <v>1167</v>
+        <v>1174</v>
       </c>
       <c r="H87" t="s">
-        <v>1347</v>
+        <v>1354</v>
       </c>
       <c r="I87" t="s">
-        <v>1432</v>
+        <v>1439</v>
       </c>
       <c r="L87" t="s">
-        <v>1507</v>
+        <v>1514</v>
       </c>
     </row>
     <row r="88" spans="6:12" x14ac:dyDescent="0.35">
       <c r="F88" t="s">
-        <v>1174</v>
+        <v>1180</v>
       </c>
       <c r="H88" t="s">
-        <v>1354</v>
+        <v>1360</v>
       </c>
       <c r="I88" t="s">
-        <v>1439</v>
+        <v>1445</v>
       </c>
       <c r="L88" t="s">
-        <v>1514</v>
+        <v>1520</v>
       </c>
     </row>
     <row r="89" spans="6:12" x14ac:dyDescent="0.35">
       <c r="F89" t="s">
-        <v>1180</v>
+        <v>1186</v>
       </c>
       <c r="H89" t="s">
-        <v>1360</v>
-      </c>
-      <c r="I89" t="s">
-        <v>1445</v>
+        <v>1366</v>
       </c>
       <c r="L89" t="s">
-        <v>1520</v>
+        <v>1526</v>
       </c>
     </row>
     <row r="90" spans="6:12" x14ac:dyDescent="0.35">
       <c r="F90" t="s">
-        <v>1186</v>
+        <v>1194</v>
       </c>
       <c r="H90" t="s">
-        <v>1366</v>
+        <v>1374</v>
       </c>
       <c r="L90" t="s">
-        <v>1526</v>
+        <v>1534</v>
       </c>
     </row>
     <row r="91" spans="6:12" x14ac:dyDescent="0.35">
       <c r="F91" t="s">
-        <v>1194</v>
+        <v>1201</v>
       </c>
       <c r="H91" t="s">
-        <v>1374</v>
+        <v>1381</v>
       </c>
       <c r="L91" t="s">
-        <v>1534</v>
+        <v>1541</v>
       </c>
     </row>
     <row r="92" spans="6:12" x14ac:dyDescent="0.35">
       <c r="F92" t="s">
-        <v>1201</v>
+        <v>1209</v>
       </c>
       <c r="H92" t="s">
-        <v>1381</v>
+        <v>1389</v>
       </c>
       <c r="L92" t="s">
-        <v>1541</v>
+        <v>1549</v>
       </c>
     </row>
     <row r="93" spans="6:12" x14ac:dyDescent="0.35">
       <c r="F93" t="s">
-        <v>1209</v>
+        <v>1216</v>
       </c>
       <c r="H93" t="s">
-        <v>1389</v>
+        <v>1396</v>
       </c>
       <c r="L93" t="s">
-        <v>1549</v>
+        <v>1556</v>
       </c>
     </row>
     <row r="94" spans="6:12" x14ac:dyDescent="0.35">
       <c r="F94" t="s">
-        <v>1216</v>
-      </c>
-      <c r="H94" t="s">
-        <v>1396</v>
-      </c>
-      <c r="L94" t="s">
-        <v>1556</v>
+        <v>1222</v>
       </c>
     </row>
     <row r="95" spans="6:12" x14ac:dyDescent="0.35">
       <c r="F95" t="s">
-        <v>1222</v>
+        <v>1230</v>
       </c>
     </row>
     <row r="96" spans="6:12" x14ac:dyDescent="0.35">
       <c r="F96" t="s">
-        <v>1230</v>
+        <v>1237</v>
       </c>
     </row>
     <row r="97" spans="6:12" x14ac:dyDescent="0.35">
       <c r="F97" t="s">
-        <v>1237</v>
+        <v>1243</v>
       </c>
     </row>
     <row r="98" spans="6:12" x14ac:dyDescent="0.35">
       <c r="F98" t="s">
-        <v>1243</v>
+        <v>1251</v>
       </c>
     </row>
     <row r="99" spans="6:12" x14ac:dyDescent="0.35">
       <c r="F99" t="s">
-        <v>1251</v>
+        <v>1258</v>
       </c>
     </row>
     <row r="100" spans="6:12" x14ac:dyDescent="0.35">
       <c r="F100" t="s">
-        <v>1258</v>
+        <v>1264</v>
       </c>
     </row>
     <row r="101" spans="6:12" x14ac:dyDescent="0.35">
       <c r="F101" t="s">
-        <v>1264</v>
+        <v>1272</v>
       </c>
     </row>
     <row r="102" spans="6:12" x14ac:dyDescent="0.35">
       <c r="F102" t="s">
-        <v>1272</v>
+        <v>1279</v>
       </c>
     </row>
     <row r="103" spans="6:12" x14ac:dyDescent="0.35">
       <c r="F103" t="s">
-        <v>1279</v>
+        <v>1285</v>
       </c>
     </row>
     <row r="104" spans="6:12" x14ac:dyDescent="0.35">
       <c r="F104" t="s">
-        <v>1285</v>
+        <v>1168</v>
+      </c>
+      <c r="H104" t="s">
+        <v>1348</v>
+      </c>
+      <c r="I104" t="s">
+        <v>1433</v>
+      </c>
+      <c r="L104" t="s">
+        <v>1508</v>
       </c>
     </row>
     <row r="105" spans="6:12" x14ac:dyDescent="0.35">
       <c r="F105" t="s">
-        <v>1168</v>
+        <v>1175</v>
       </c>
       <c r="H105" t="s">
-        <v>1348</v>
+        <v>1355</v>
       </c>
       <c r="I105" t="s">
-        <v>1433</v>
+        <v>1440</v>
       </c>
       <c r="L105" t="s">
-        <v>1508</v>
+        <v>1515</v>
       </c>
     </row>
     <row r="106" spans="6:12" x14ac:dyDescent="0.35">
       <c r="F106" t="s">
-        <v>1175</v>
+        <v>1181</v>
       </c>
       <c r="H106" t="s">
-        <v>1355</v>
+        <v>1361</v>
       </c>
       <c r="I106" t="s">
-        <v>1440</v>
+        <v>1446</v>
       </c>
       <c r="L106" t="s">
-        <v>1515</v>
+        <v>1521</v>
       </c>
     </row>
     <row r="107" spans="6:12" x14ac:dyDescent="0.35">
       <c r="F107" t="s">
-        <v>1181</v>
+        <v>1187</v>
       </c>
       <c r="H107" t="s">
-        <v>1361</v>
-      </c>
-      <c r="I107" t="s">
-        <v>1446</v>
+        <v>1367</v>
       </c>
       <c r="L107" t="s">
-        <v>1521</v>
+        <v>1527</v>
       </c>
     </row>
     <row r="108" spans="6:12" x14ac:dyDescent="0.35">
       <c r="F108" t="s">
-        <v>1187</v>
+        <v>1195</v>
       </c>
       <c r="H108" t="s">
-        <v>1367</v>
+        <v>1375</v>
       </c>
       <c r="L108" t="s">
-        <v>1527</v>
+        <v>1535</v>
       </c>
     </row>
     <row r="109" spans="6:12" x14ac:dyDescent="0.35">
       <c r="F109" t="s">
-        <v>1195</v>
+        <v>1202</v>
       </c>
       <c r="H109" t="s">
-        <v>1375</v>
+        <v>1382</v>
       </c>
       <c r="L109" t="s">
-        <v>1535</v>
+        <v>1542</v>
       </c>
     </row>
     <row r="110" spans="6:12" x14ac:dyDescent="0.35">
       <c r="F110" t="s">
-        <v>1202</v>
+        <v>1210</v>
       </c>
       <c r="H110" t="s">
-        <v>1382</v>
+        <v>1390</v>
       </c>
       <c r="L110" t="s">
-        <v>1542</v>
+        <v>1550</v>
       </c>
     </row>
     <row r="111" spans="6:12" x14ac:dyDescent="0.35">
       <c r="F111" t="s">
-        <v>1210</v>
-      </c>
-      <c r="H111" t="s">
-        <v>1390</v>
+        <v>1217</v>
       </c>
       <c r="L111" t="s">
-        <v>1550</v>
+        <v>1557</v>
       </c>
     </row>
     <row r="112" spans="6:12" x14ac:dyDescent="0.35">
       <c r="F112" t="s">
-        <v>1217</v>
-      </c>
-      <c r="L112" t="s">
-        <v>1557</v>
+        <v>1223</v>
       </c>
     </row>
     <row r="113" spans="6:14" x14ac:dyDescent="0.35">
       <c r="F113" t="s">
-        <v>1223</v>
+        <v>1231</v>
       </c>
     </row>
     <row r="114" spans="6:14" x14ac:dyDescent="0.35">
       <c r="F114" t="s">
-        <v>1231</v>
+        <v>1238</v>
       </c>
     </row>
     <row r="115" spans="6:14" x14ac:dyDescent="0.35">
       <c r="F115" t="s">
-        <v>1238</v>
+        <v>1244</v>
       </c>
     </row>
     <row r="116" spans="6:14" x14ac:dyDescent="0.35">
       <c r="F116" t="s">
-        <v>1244</v>
+        <v>1252</v>
       </c>
     </row>
     <row r="117" spans="6:14" x14ac:dyDescent="0.35">
       <c r="F117" t="s">
-        <v>1252</v>
+        <v>1259</v>
       </c>
     </row>
     <row r="118" spans="6:14" x14ac:dyDescent="0.35">
       <c r="F118" t="s">
-        <v>1259</v>
+        <v>1265</v>
       </c>
     </row>
     <row r="119" spans="6:14" x14ac:dyDescent="0.35">
       <c r="F119" t="s">
-        <v>1265</v>
+        <v>1273</v>
       </c>
     </row>
     <row r="120" spans="6:14" x14ac:dyDescent="0.35">
       <c r="F120" t="s">
-        <v>1273</v>
+        <v>1280</v>
       </c>
     </row>
     <row r="121" spans="6:14" x14ac:dyDescent="0.35">
       <c r="F121" t="s">
-        <v>1280</v>
+        <v>1286</v>
       </c>
     </row>
     <row r="122" spans="6:14" x14ac:dyDescent="0.35">
       <c r="F122" t="s">
-        <v>1286</v>
+        <v>1154</v>
+      </c>
+      <c r="G122" t="s">
+        <v>1310</v>
+      </c>
+      <c r="H122" t="s">
+        <v>1334</v>
+      </c>
+      <c r="I122" t="s">
+        <v>1419</v>
+      </c>
+      <c r="L122" t="s">
+        <v>1494</v>
+      </c>
+      <c r="M122" t="s">
+        <v>1582</v>
       </c>
     </row>
     <row r="123" spans="6:14" x14ac:dyDescent="0.35">
       <c r="F123" t="s">
-        <v>1154</v>
-      </c>
-      <c r="G123" t="s">
-        <v>1310</v>
+        <v>1159</v>
       </c>
       <c r="H123" t="s">
-        <v>1334</v>
+        <v>1339</v>
       </c>
       <c r="I123" t="s">
-        <v>1419</v>
+        <v>1424</v>
       </c>
       <c r="L123" t="s">
-        <v>1494</v>
-      </c>
-      <c r="M123" t="s">
-        <v>1582</v>
+        <v>1499</v>
       </c>
     </row>
     <row r="124" spans="6:14" x14ac:dyDescent="0.35">
       <c r="F124" t="s">
-        <v>1159</v>
+        <v>1149</v>
+      </c>
+      <c r="G124" t="s">
+        <v>1305</v>
       </c>
       <c r="H124" t="s">
-        <v>1339</v>
+        <v>1329</v>
       </c>
       <c r="I124" t="s">
-        <v>1424</v>
+        <v>1414</v>
       </c>
       <c r="L124" t="s">
-        <v>1499</v>
+        <v>1489</v>
+      </c>
+      <c r="M124" t="s">
+        <v>1577</v>
+      </c>
+      <c r="N124" t="s">
+        <v>1593</v>
       </c>
     </row>
     <row r="125" spans="6:14" x14ac:dyDescent="0.35">
       <c r="F125" t="s">
-        <v>1149</v>
+        <v>1144</v>
       </c>
       <c r="G125" t="s">
-        <v>1305</v>
+        <v>1300</v>
       </c>
       <c r="H125" t="s">
-        <v>1329</v>
+        <v>1324</v>
       </c>
       <c r="I125" t="s">
-        <v>1414</v>
+        <v>1409</v>
+      </c>
+      <c r="J125" t="s">
+        <v>1462</v>
       </c>
       <c r="L125" t="s">
-        <v>1489</v>
+        <v>1484</v>
       </c>
       <c r="M125" t="s">
-        <v>1577</v>
+        <v>1572</v>
       </c>
       <c r="N125" t="s">
-        <v>1593</v>
+        <v>1588</v>
       </c>
     </row>
     <row r="126" spans="6:14" x14ac:dyDescent="0.35">
       <c r="F126" t="s">
-        <v>1144</v>
+        <v>1134</v>
       </c>
       <c r="G126" t="s">
-        <v>1300</v>
+        <v>1290</v>
       </c>
       <c r="H126" t="s">
-        <v>1324</v>
+        <v>1314</v>
       </c>
       <c r="I126" t="s">
-        <v>1409</v>
+        <v>1399</v>
       </c>
       <c r="J126" t="s">
-        <v>1462</v>
+        <v>1452</v>
+      </c>
+      <c r="K126" t="s">
+        <v>1467</v>
       </c>
       <c r="L126" t="s">
-        <v>1484</v>
+        <v>1474</v>
       </c>
       <c r="M126" t="s">
-        <v>1572</v>
+        <v>1562</v>
       </c>
       <c r="N126" t="s">
-        <v>1588</v>
+        <v>1189</v>
       </c>
     </row>
     <row r="127" spans="6:14" x14ac:dyDescent="0.35">
       <c r="F127" t="s">
-        <v>1134</v>
+        <v>1139</v>
       </c>
       <c r="G127" t="s">
-        <v>1290</v>
+        <v>1295</v>
       </c>
       <c r="H127" t="s">
-        <v>1314</v>
+        <v>1319</v>
       </c>
       <c r="I127" t="s">
-        <v>1399</v>
+        <v>1404</v>
       </c>
       <c r="J127" t="s">
-        <v>1452</v>
-      </c>
-      <c r="K127" t="s">
-        <v>1467</v>
+        <v>1457</v>
       </c>
       <c r="L127" t="s">
-        <v>1474</v>
+        <v>1479</v>
       </c>
       <c r="M127" t="s">
-        <v>1562</v>
+        <v>1567</v>
       </c>
       <c r="N127" t="s">
-        <v>1189</v>
+        <v>1194</v>
       </c>
     </row>
     <row r="128" spans="6:14" x14ac:dyDescent="0.35">
       <c r="F128" t="s">
-        <v>1139</v>
+        <v>1155</v>
       </c>
       <c r="G128" t="s">
-        <v>1295</v>
+        <v>1311</v>
       </c>
       <c r="H128" t="s">
-        <v>1319</v>
+        <v>1335</v>
       </c>
       <c r="I128" t="s">
-        <v>1404</v>
-      </c>
-      <c r="J128" t="s">
-        <v>1457</v>
+        <v>1420</v>
       </c>
       <c r="L128" t="s">
-        <v>1479</v>
+        <v>1495</v>
       </c>
       <c r="M128" t="s">
-        <v>1567</v>
-      </c>
-      <c r="N128" t="s">
-        <v>1194</v>
+        <v>1583</v>
       </c>
     </row>
     <row r="129" spans="6:14" x14ac:dyDescent="0.35">
       <c r="F129" t="s">
-        <v>1155</v>
-      </c>
-      <c r="G129" t="s">
-        <v>1311</v>
+        <v>1160</v>
       </c>
       <c r="H129" t="s">
-        <v>1335</v>
+        <v>1340</v>
       </c>
       <c r="I129" t="s">
-        <v>1420</v>
+        <v>1425</v>
       </c>
       <c r="L129" t="s">
-        <v>1495</v>
-      </c>
-      <c r="M129" t="s">
-        <v>1583</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="130" spans="6:14" x14ac:dyDescent="0.35">
       <c r="F130" t="s">
-        <v>1160</v>
+        <v>1150</v>
+      </c>
+      <c r="G130" t="s">
+        <v>1306</v>
       </c>
       <c r="H130" t="s">
-        <v>1340</v>
+        <v>1330</v>
       </c>
       <c r="I130" t="s">
-        <v>1425</v>
+        <v>1415</v>
       </c>
       <c r="L130" t="s">
-        <v>1500</v>
+        <v>1490</v>
+      </c>
+      <c r="M130" t="s">
+        <v>1578</v>
+      </c>
+      <c r="N130" t="s">
+        <v>1594</v>
       </c>
     </row>
     <row r="131" spans="6:14" x14ac:dyDescent="0.35">
       <c r="F131" t="s">
-        <v>1150</v>
+        <v>1145</v>
       </c>
       <c r="G131" t="s">
-        <v>1306</v>
+        <v>1301</v>
       </c>
       <c r="H131" t="s">
-        <v>1330</v>
+        <v>1325</v>
       </c>
       <c r="I131" t="s">
-        <v>1415</v>
+        <v>1410</v>
+      </c>
+      <c r="J131" t="s">
+        <v>1463</v>
       </c>
       <c r="L131" t="s">
-        <v>1490</v>
+        <v>1485</v>
       </c>
       <c r="M131" t="s">
-        <v>1578</v>
+        <v>1573</v>
       </c>
       <c r="N131" t="s">
-        <v>1594</v>
+        <v>1589</v>
       </c>
     </row>
     <row r="132" spans="6:14" x14ac:dyDescent="0.35">
       <c r="F132" t="s">
-        <v>1145</v>
+        <v>1135</v>
       </c>
       <c r="G132" t="s">
-        <v>1301</v>
+        <v>1291</v>
       </c>
       <c r="H132" t="s">
-        <v>1325</v>
+        <v>1315</v>
       </c>
       <c r="I132" t="s">
-        <v>1410</v>
+        <v>1400</v>
       </c>
       <c r="J132" t="s">
-        <v>1463</v>
+        <v>1453</v>
+      </c>
+      <c r="K132" t="s">
+        <v>1468</v>
       </c>
       <c r="L132" t="s">
-        <v>1485</v>
+        <v>1475</v>
       </c>
       <c r="M132" t="s">
-        <v>1573</v>
+        <v>1563</v>
       </c>
       <c r="N132" t="s">
-        <v>1589</v>
+        <v>1190</v>
       </c>
     </row>
     <row r="133" spans="6:14" x14ac:dyDescent="0.35">
       <c r="F133" t="s">
-        <v>1135</v>
+        <v>1140</v>
       </c>
       <c r="G133" t="s">
-        <v>1291</v>
+        <v>1296</v>
       </c>
       <c r="H133" t="s">
-        <v>1315</v>
+        <v>1320</v>
       </c>
       <c r="I133" t="s">
-        <v>1400</v>
+        <v>1405</v>
       </c>
       <c r="J133" t="s">
-        <v>1453</v>
-      </c>
-      <c r="K133" t="s">
-        <v>1468</v>
+        <v>1458</v>
       </c>
       <c r="L133" t="s">
-        <v>1475</v>
+        <v>1480</v>
       </c>
       <c r="M133" t="s">
-        <v>1563</v>
+        <v>1568</v>
       </c>
       <c r="N133" t="s">
-        <v>1190</v>
+        <v>1195</v>
       </c>
     </row>
     <row r="134" spans="6:14" x14ac:dyDescent="0.35">
       <c r="F134" t="s">
-        <v>1140</v>
-      </c>
-      <c r="G134" t="s">
-        <v>1296</v>
+        <v>1169</v>
       </c>
       <c r="H134" t="s">
-        <v>1320</v>
+        <v>1349</v>
       </c>
       <c r="I134" t="s">
-        <v>1405</v>
-      </c>
-      <c r="J134" t="s">
-        <v>1458</v>
+        <v>1434</v>
       </c>
       <c r="L134" t="s">
-        <v>1480</v>
-      </c>
-      <c r="M134" t="s">
-        <v>1568</v>
-      </c>
-      <c r="N134" t="s">
-        <v>1195</v>
+        <v>1509</v>
       </c>
     </row>
     <row r="135" spans="6:14" x14ac:dyDescent="0.35">
       <c r="F135" t="s">
-        <v>1169</v>
+        <v>1176</v>
       </c>
       <c r="H135" t="s">
-        <v>1349</v>
+        <v>1356</v>
       </c>
       <c r="I135" t="s">
-        <v>1434</v>
+        <v>1441</v>
       </c>
       <c r="L135" t="s">
-        <v>1509</v>
+        <v>1516</v>
       </c>
     </row>
     <row r="136" spans="6:14" x14ac:dyDescent="0.35">
       <c r="F136" t="s">
-        <v>1176</v>
+        <v>1182</v>
       </c>
       <c r="H136" t="s">
-        <v>1356</v>
+        <v>1362</v>
       </c>
       <c r="I136" t="s">
-        <v>1441</v>
+        <v>1447</v>
       </c>
       <c r="L136" t="s">
-        <v>1516</v>
+        <v>1522</v>
       </c>
     </row>
     <row r="137" spans="6:14" x14ac:dyDescent="0.35">
       <c r="F137" t="s">
-        <v>1182</v>
+        <v>1188</v>
       </c>
       <c r="H137" t="s">
-        <v>1362</v>
-      </c>
-      <c r="I137" t="s">
-        <v>1447</v>
+        <v>1368</v>
       </c>
       <c r="L137" t="s">
-        <v>1522</v>
+        <v>1528</v>
       </c>
     </row>
     <row r="138" spans="6:14" x14ac:dyDescent="0.35">
       <c r="F138" t="s">
-        <v>1188</v>
+        <v>1196</v>
       </c>
       <c r="H138" t="s">
-        <v>1368</v>
+        <v>1376</v>
       </c>
       <c r="L138" t="s">
-        <v>1528</v>
+        <v>1536</v>
       </c>
     </row>
     <row r="139" spans="6:14" x14ac:dyDescent="0.35">
       <c r="F139" t="s">
-        <v>1196</v>
+        <v>1203</v>
       </c>
       <c r="H139" t="s">
-        <v>1376</v>
+        <v>1383</v>
       </c>
       <c r="L139" t="s">
-        <v>1536</v>
+        <v>1543</v>
       </c>
     </row>
     <row r="140" spans="6:14" x14ac:dyDescent="0.35">
       <c r="F140" t="s">
-        <v>1203</v>
+        <v>1211</v>
       </c>
       <c r="H140" t="s">
-        <v>1383</v>
+        <v>1391</v>
       </c>
       <c r="L140" t="s">
-        <v>1543</v>
+        <v>1551</v>
       </c>
     </row>
     <row r="141" spans="6:14" x14ac:dyDescent="0.35">
       <c r="F141" t="s">
-        <v>1211</v>
-      </c>
-      <c r="H141" t="s">
-        <v>1391</v>
+        <v>1218</v>
       </c>
       <c r="L141" t="s">
-        <v>1551</v>
+        <v>1558</v>
       </c>
     </row>
     <row r="142" spans="6:14" x14ac:dyDescent="0.35">
       <c r="F142" t="s">
-        <v>1218</v>
-      </c>
-      <c r="L142" t="s">
-        <v>1558</v>
+        <v>1224</v>
       </c>
     </row>
     <row r="143" spans="6:14" x14ac:dyDescent="0.35">
       <c r="F143" t="s">
-        <v>1224</v>
+        <v>1232</v>
       </c>
     </row>
     <row r="144" spans="6:14" x14ac:dyDescent="0.35">
       <c r="F144" t="s">
-        <v>1232</v>
+        <v>1239</v>
       </c>
     </row>
     <row r="145" spans="6:14" x14ac:dyDescent="0.35">
       <c r="F145" t="s">
-        <v>1239</v>
+        <v>1245</v>
       </c>
     </row>
     <row r="146" spans="6:14" x14ac:dyDescent="0.35">
       <c r="F146" t="s">
-        <v>1245</v>
+        <v>1253</v>
       </c>
     </row>
     <row r="147" spans="6:14" x14ac:dyDescent="0.35">
       <c r="F147" t="s">
-        <v>1253</v>
+        <v>1260</v>
       </c>
     </row>
     <row r="148" spans="6:14" x14ac:dyDescent="0.35">
       <c r="F148" t="s">
-        <v>1260</v>
+        <v>1266</v>
       </c>
     </row>
     <row r="149" spans="6:14" x14ac:dyDescent="0.35">
       <c r="F149" t="s">
-        <v>1266</v>
+        <v>1274</v>
       </c>
     </row>
     <row r="150" spans="6:14" x14ac:dyDescent="0.35">
       <c r="F150" t="s">
-        <v>1274</v>
+        <v>1281</v>
       </c>
     </row>
     <row r="151" spans="6:14" x14ac:dyDescent="0.35">
       <c r="F151" t="s">
-        <v>1281</v>
+        <v>1287</v>
       </c>
     </row>
     <row r="152" spans="6:14" x14ac:dyDescent="0.35">
       <c r="F152" t="s">
-        <v>1287</v>
+        <v>1156</v>
+      </c>
+      <c r="H152" t="s">
+        <v>1336</v>
+      </c>
+      <c r="I152" t="s">
+        <v>1421</v>
+      </c>
+      <c r="L152" t="s">
+        <v>1496</v>
+      </c>
+      <c r="M152" t="s">
+        <v>1584</v>
       </c>
     </row>
     <row r="153" spans="6:14" x14ac:dyDescent="0.35">
       <c r="F153" t="s">
-        <v>1156</v>
+        <v>1161</v>
       </c>
       <c r="H153" t="s">
-        <v>1336</v>
+        <v>1341</v>
       </c>
       <c r="I153" t="s">
-        <v>1421</v>
+        <v>1426</v>
       </c>
       <c r="L153" t="s">
-        <v>1496</v>
-      </c>
-      <c r="M153" t="s">
-        <v>1584</v>
+        <v>1501</v>
       </c>
     </row>
     <row r="154" spans="6:14" x14ac:dyDescent="0.35">
       <c r="F154" t="s">
-        <v>1161</v>
+        <v>1151</v>
+      </c>
+      <c r="G154" t="s">
+        <v>1307</v>
       </c>
       <c r="H154" t="s">
-        <v>1341</v>
+        <v>1331</v>
       </c>
       <c r="I154" t="s">
-        <v>1426</v>
+        <v>1416</v>
       </c>
       <c r="L154" t="s">
-        <v>1501</v>
+        <v>1491</v>
+      </c>
+      <c r="M154" t="s">
+        <v>1579</v>
+      </c>
+      <c r="N154" t="s">
+        <v>1595</v>
       </c>
     </row>
     <row r="155" spans="6:14" x14ac:dyDescent="0.35">
       <c r="F155" t="s">
-        <v>1151</v>
+        <v>1146</v>
       </c>
       <c r="G155" t="s">
-        <v>1307</v>
+        <v>1302</v>
       </c>
       <c r="H155" t="s">
-        <v>1331</v>
+        <v>1326</v>
       </c>
       <c r="I155" t="s">
-        <v>1416</v>
+        <v>1411</v>
+      </c>
+      <c r="J155" t="s">
+        <v>1464</v>
       </c>
       <c r="L155" t="s">
-        <v>1491</v>
+        <v>1486</v>
       </c>
       <c r="M155" t="s">
-        <v>1579</v>
+        <v>1574</v>
       </c>
       <c r="N155" t="s">
-        <v>1595</v>
+        <v>1590</v>
       </c>
     </row>
     <row r="156" spans="6:14" x14ac:dyDescent="0.35">
       <c r="F156" t="s">
-        <v>1146</v>
+        <v>1136</v>
       </c>
       <c r="G156" t="s">
-        <v>1302</v>
+        <v>1292</v>
       </c>
       <c r="H156" t="s">
-        <v>1326</v>
+        <v>1316</v>
       </c>
       <c r="I156" t="s">
-        <v>1411</v>
+        <v>1401</v>
       </c>
       <c r="J156" t="s">
-        <v>1464</v>
+        <v>1454</v>
+      </c>
+      <c r="K156" t="s">
+        <v>1469</v>
       </c>
       <c r="L156" t="s">
-        <v>1486</v>
+        <v>1476</v>
       </c>
       <c r="M156" t="s">
-        <v>1574</v>
+        <v>1564</v>
       </c>
       <c r="N156" t="s">
-        <v>1590</v>
+        <v>1191</v>
       </c>
     </row>
     <row r="157" spans="6:14" x14ac:dyDescent="0.35">
       <c r="F157" t="s">
-        <v>1136</v>
+        <v>1141</v>
       </c>
       <c r="G157" t="s">
-        <v>1292</v>
+        <v>1297</v>
       </c>
       <c r="H157" t="s">
-        <v>1316</v>
+        <v>1321</v>
       </c>
       <c r="I157" t="s">
-        <v>1401</v>
+        <v>1406</v>
       </c>
       <c r="J157" t="s">
-        <v>1454</v>
-      </c>
-      <c r="K157" t="s">
-        <v>1469</v>
+        <v>1459</v>
       </c>
       <c r="L157" t="s">
-        <v>1476</v>
+        <v>1481</v>
       </c>
       <c r="M157" t="s">
-        <v>1564</v>
+        <v>1569</v>
       </c>
       <c r="N157" t="s">
-        <v>1191</v>
-      </c>
-    </row>
-    <row r="158" spans="6:14" x14ac:dyDescent="0.35">
-      <c r="F158" t="s">
-        <v>1141</v>
-      </c>
-      <c r="G158" t="s">
-        <v>1297</v>
-      </c>
-      <c r="H158" t="s">
-        <v>1321</v>
-      </c>
-      <c r="I158" t="s">
-        <v>1406</v>
-      </c>
-      <c r="J158" t="s">
-        <v>1459</v>
-      </c>
-      <c r="L158" t="s">
-        <v>1481</v>
-      </c>
-      <c r="M158" t="s">
-        <v>1569</v>
-      </c>
-      <c r="N158" t="s">
         <v>1196</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="F2:N158" xr:uid="{75E7CC39-AA01-4AB9-B162-02F569063FA9}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="F3:N158">
-      <sortCondition ref="F2:F158"/>
+  <autoFilter ref="F1:N157" xr:uid="{75E7CC39-AA01-4AB9-B162-02F569063FA9}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="F2:N157">
+      <sortCondition ref="F1:F157"/>
     </sortState>
   </autoFilter>
   <phoneticPr fontId="2" type="noConversion"/>
@@ -9688,253 +9700,251 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6EACFF71-F93F-43B9-8608-0ACFAF57A8D1}">
-  <dimension ref="B3:J14"/>
+  <dimension ref="A1:I12"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="21.1796875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="18" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="15.26953125" bestFit="1" customWidth="1"/>
-    <col min="6" max="10" width="21.1796875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="21.1796875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18" bestFit="1" customWidth="1"/>
+    <col min="3" max="9" width="21.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B3" s="5" t="s">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="C3" s="5" t="s">
+      <c r="B1" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="D3" s="5" t="s">
+      <c r="C1" s="5" t="s">
         <v>129</v>
       </c>
-      <c r="E3" s="5" t="s">
+      <c r="D1" s="5" t="s">
         <v>185</v>
       </c>
-      <c r="F3" s="5" t="s">
+      <c r="E1" s="5" t="s">
         <v>249</v>
       </c>
-      <c r="G3" s="5" t="s">
+      <c r="F1" s="5" t="s">
         <v>262</v>
       </c>
-      <c r="H3" s="5" t="s">
+      <c r="G1" s="5" t="s">
         <v>265</v>
       </c>
-      <c r="I3" s="5" t="s">
+      <c r="H1" s="5" t="s">
         <v>307</v>
       </c>
-      <c r="J3" s="5" t="s">
+      <c r="I1" s="5" t="s">
         <v>310</v>
       </c>
     </row>
-    <row r="4" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B4" t="s">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
         <v>313</v>
       </c>
+      <c r="B2" t="s">
+        <v>738</v>
+      </c>
+      <c r="C2" t="s">
+        <v>313</v>
+      </c>
+      <c r="D2" t="s">
+        <v>313</v>
+      </c>
+      <c r="E2" t="s">
+        <v>313</v>
+      </c>
+      <c r="F2" t="s">
+        <v>315</v>
+      </c>
+      <c r="G2" t="s">
+        <v>315</v>
+      </c>
+      <c r="H2" t="s">
+        <v>313</v>
+      </c>
+      <c r="I2" t="s">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>317</v>
+      </c>
+      <c r="C3" t="s">
+        <v>315</v>
+      </c>
+      <c r="D3" t="s">
+        <v>315</v>
+      </c>
+      <c r="E3" t="s">
+        <v>315</v>
+      </c>
+      <c r="F3" t="s">
+        <v>319</v>
+      </c>
+      <c r="G3" t="s">
+        <v>1600</v>
+      </c>
+      <c r="H3" t="s">
+        <v>315</v>
+      </c>
+      <c r="I3" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>319</v>
+      </c>
       <c r="C4" t="s">
+        <v>736</v>
+      </c>
+      <c r="D4" t="s">
+        <v>736</v>
+      </c>
+      <c r="E4" t="s">
+        <v>736</v>
+      </c>
+      <c r="F4" t="s">
         <v>738</v>
       </c>
-      <c r="D4" t="s">
-        <v>313</v>
-      </c>
-      <c r="E4" t="s">
-        <v>313</v>
-      </c>
-      <c r="F4" t="s">
-        <v>313</v>
-      </c>
       <c r="G4" t="s">
-        <v>315</v>
+        <v>738</v>
       </c>
       <c r="H4" t="s">
-        <v>315</v>
+        <v>736</v>
       </c>
       <c r="I4" t="s">
-        <v>313</v>
-      </c>
-      <c r="J4" t="s">
-        <v>313</v>
-      </c>
-    </row>
-    <row r="5" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B5" t="s">
-        <v>317</v>
+        <v>1600</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>1598</v>
+      </c>
+      <c r="C5" t="s">
+        <v>314</v>
       </c>
       <c r="D5" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="E5" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="F5" t="s">
-        <v>315</v>
+        <v>318</v>
       </c>
       <c r="G5" t="s">
+        <v>314</v>
+      </c>
+      <c r="H5" t="s">
+        <v>314</v>
+      </c>
+      <c r="I5" t="s">
+        <v>736</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>736</v>
+      </c>
+      <c r="C6" t="s">
+        <v>738</v>
+      </c>
+      <c r="D6" t="s">
+        <v>738</v>
+      </c>
+      <c r="E6" t="s">
+        <v>738</v>
+      </c>
+      <c r="G6" t="s">
         <v>319</v>
-      </c>
-      <c r="H5" t="s">
-        <v>1600</v>
-      </c>
-      <c r="I5" t="s">
-        <v>315</v>
-      </c>
-      <c r="J5" t="s">
-        <v>315</v>
-      </c>
-    </row>
-    <row r="6" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B6" t="s">
-        <v>319</v>
-      </c>
-      <c r="D6" t="s">
-        <v>736</v>
-      </c>
-      <c r="E6" t="s">
-        <v>736</v>
-      </c>
-      <c r="F6" t="s">
-        <v>736</v>
-      </c>
-      <c r="G6" t="s">
-        <v>738</v>
       </c>
       <c r="H6" t="s">
         <v>738</v>
       </c>
       <c r="I6" t="s">
-        <v>736</v>
-      </c>
-      <c r="J6" t="s">
-        <v>1600</v>
-      </c>
-    </row>
-    <row r="7" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B7" t="s">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>314</v>
+      </c>
+      <c r="C7" t="s">
+        <v>1599</v>
+      </c>
+      <c r="D7" t="s">
+        <v>1599</v>
+      </c>
+      <c r="E7" t="s">
+        <v>1599</v>
+      </c>
+      <c r="G7" t="s">
+        <v>738</v>
+      </c>
+      <c r="H7" t="s">
+        <v>1599</v>
+      </c>
+      <c r="I7" t="s">
         <v>1598</v>
       </c>
-      <c r="D7" t="s">
-        <v>314</v>
-      </c>
-      <c r="E7" t="s">
-        <v>314</v>
-      </c>
-      <c r="F7" t="s">
-        <v>314</v>
-      </c>
-      <c r="G7" t="s">
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>739</v>
+      </c>
+      <c r="C8" t="s">
         <v>318</v>
       </c>
-      <c r="H7" t="s">
-        <v>314</v>
-      </c>
-      <c r="I7" t="s">
-        <v>314</v>
-      </c>
-      <c r="J7" t="s">
-        <v>736</v>
-      </c>
-    </row>
-    <row r="8" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B8" t="s">
-        <v>736</v>
-      </c>
       <c r="D8" t="s">
+        <v>318</v>
+      </c>
+      <c r="E8" t="s">
+        <v>318</v>
+      </c>
+      <c r="G8" t="s">
+        <v>1601</v>
+      </c>
+      <c r="H8" t="s">
+        <v>318</v>
+      </c>
+      <c r="I8" t="s">
+        <v>1602</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
         <v>738</v>
       </c>
-      <c r="E8" t="s">
+      <c r="G9" t="s">
+        <v>318</v>
+      </c>
+      <c r="I9" t="s">
         <v>738</v>
       </c>
-      <c r="F8" t="s">
-        <v>738</v>
-      </c>
-      <c r="H8" t="s">
-        <v>319</v>
-      </c>
-      <c r="I8" t="s">
-        <v>738</v>
-      </c>
-      <c r="J8" t="s">
-        <v>314</v>
-      </c>
-    </row>
-    <row r="9" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B9" t="s">
-        <v>314</v>
-      </c>
-      <c r="D9" t="s">
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>315</v>
+      </c>
+      <c r="G10" t="s">
         <v>1599</v>
       </c>
-      <c r="E9" t="s">
+      <c r="I10" t="s">
         <v>1599</v>
       </c>
-      <c r="F9" t="s">
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
         <v>1599</v>
       </c>
-      <c r="H9" t="s">
-        <v>738</v>
-      </c>
-      <c r="I9" t="s">
-        <v>1599</v>
-      </c>
-      <c r="J9" t="s">
-        <v>1598</v>
-      </c>
-    </row>
-    <row r="10" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B10" t="s">
-        <v>739</v>
-      </c>
-      <c r="D10" t="s">
+      <c r="I11" t="s">
         <v>318</v>
       </c>
-      <c r="E10" t="s">
-        <v>318</v>
-      </c>
-      <c r="F10" t="s">
-        <v>318</v>
-      </c>
-      <c r="H10" t="s">
-        <v>1601</v>
-      </c>
-      <c r="I10" t="s">
-        <v>318</v>
-      </c>
-      <c r="J10" t="s">
-        <v>1602</v>
-      </c>
-    </row>
-    <row r="11" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B11" t="s">
-        <v>738</v>
-      </c>
-      <c r="H11" t="s">
-        <v>318</v>
-      </c>
-      <c r="J11" t="s">
-        <v>738</v>
-      </c>
-    </row>
-    <row r="12" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B12" t="s">
-        <v>315</v>
-      </c>
-      <c r="H12" t="s">
-        <v>1599</v>
-      </c>
-      <c r="J12" t="s">
-        <v>1599</v>
-      </c>
-    </row>
-    <row r="13" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B13" t="s">
-        <v>1599</v>
-      </c>
-      <c r="J13" t="s">
-        <v>318</v>
-      </c>
-    </row>
-    <row r="14" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B14" t="s">
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
         <v>318</v>
       </c>
     </row>
@@ -9949,10 +9959,9 @@
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="6" max="6" width="11.1796875" bestFit="1" customWidth="1"/>
-    <col min="7" max="10" width="9.6328125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="10.1796875" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8.90625" customWidth="1"/>
-    <col min="13" max="14" width="9.6328125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.6328125" customWidth="1"/>
+    <col min="8" max="13" width="12.36328125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="12.36328125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="7:14" x14ac:dyDescent="0.35">

</xml_diff>